<commit_message>
feat: add decorative title banner to lead import template
Row 1 is now a merged "SEIKI — Modèle d'import de leads" banner,
headers moved to row 2, data starts row 3. parseFile/segment dropdown
updated to match.
</commit_message>
<xml_diff>
--- a/public/templates/leads-import-template.xlsx
+++ b/public/templates/leads-import-template.xlsx
@@ -11,7 +11,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+  <si>
+    <t>SEIKI — Modèle d'import de leads</t>
+  </si>
   <si>
     <t>Nom de la société</t>
   </si>
@@ -77,7 +80,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -87,14 +90,24 @@
     </font>
     <font>
       <b/>
+      <color rgb="FFD4C4A8"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF141414"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -109,9 +122,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -451,79 +467,96 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="10" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+    </row>
+    <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="J2" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
+      <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="E2" t="s">
+      <c r="D3" t="s">
         <v>14</v>
       </c>
-      <c r="F2" t="s">
+      <c r="E3" t="s">
         <v>15</v>
       </c>
-      <c r="G2" t="s">
+      <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="H2" t="s">
+      <c r="G3" t="s">
         <v>17</v>
       </c>
-      <c r="I2" t="s">
+      <c r="H3" t="s">
         <v>18</v>
       </c>
-      <c r="J2" t="s">
+      <c r="I3" t="s">
         <v>19</v>
+      </c>
+      <c r="J3" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Segment invalide" error="Merci de choisir Media, Retail ou Instit." sqref="B2:B1000">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Segment invalide" error="Merci de choisir Media, Retail ou Instit." sqref="B3:B1000">
       <formula1>"Media,Retail,Instit"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: split lead import's contact column into Genre/Prénom/Nom
Matches the manual Add Lead form's field structure instead of a single
free-text "Nom du contact" column. contact_name is now composed via
the same formatContactName() helper the manual form already uses.
</commit_message>
<xml_diff>
--- a/public/templates/leads-import-template.xlsx
+++ b/public/templates/leads-import-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>SEIKI — Modèle d'import de leads</t>
   </si>
@@ -19,12 +19,18 @@
     <t>Nom de la société</t>
   </si>
   <si>
+    <t>Genre</t>
+  </si>
+  <si>
+    <t>Prénom</t>
+  </si>
+  <si>
+    <t>Nom</t>
+  </si>
+  <si>
     <t>Segment</t>
   </si>
   <si>
-    <t>Nom du contact</t>
-  </si>
-  <si>
     <t>Email</t>
   </si>
   <si>
@@ -49,10 +55,16 @@
     <t>Acme Corp</t>
   </si>
   <si>
+    <t>M.</t>
+  </si>
+  <si>
+    <t>Jean</t>
+  </si>
+  <si>
+    <t>DUPONT</t>
+  </si>
+  <si>
     <t>Retail</t>
-  </si>
-  <si>
-    <t>Jean Dupont</t>
   </si>
   <si>
     <t>jean.dupont@acme.com</t>
@@ -467,13 +479,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="10" width="24" customWidth="1"/>
+    <col min="1" max="12" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -486,8 +498,10 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -518,45 +532,57 @@
       <c r="J2" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="K2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="J3" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="K3" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Segment invalide" error="Merci de choisir Media, Retail ou Instit." sqref="B3:B1000">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Segment invalide" error="Merci de choisir Media, Retail ou Instit." sqref="E3:E1000">
       <formula1>"Media,Retail,Instit"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: restrict lead import's Genre column to M./Mme/Autre
Same dropdown-and-reject-invalid treatment as Segment, but optional
(blank allowed) since Genre isn't required on the manual form either.

Also fixes AddLead's toggle test to match the toggle label ("Import
Excel"), which had been updated in the working tree since the last
commit but not the test.
</commit_message>
<xml_diff>
--- a/public/templates/leads-import-template.xlsx
+++ b/public/templates/leads-import-template.xlsx
@@ -581,7 +581,10 @@
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Genre invalide" error="Merci de choisir M., Mme ou Autre (ou laisser vide)." sqref="B3:B1000">
+      <formula1>"M.,Mme,Autre"</formula1>
+    </dataValidation>
     <dataValidation type="list" showErrorMessage="1" errorTitle="Segment invalide" error="Merci de choisir Media, Retail ou Instit." sqref="E3:E1000">
       <formula1>"Media,Retail,Instit"</formula1>
     </dataValidation>

</xml_diff>